<commit_message>
Doc changes and new files for HMBv4_2_3
</commit_message>
<xml_diff>
--- a/Doc/GPIO compare.xlsx
+++ b/Doc/GPIO compare.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\BothRS485Heishamon\original\DOC_tmp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\PlatformIO_GIT\HeishaMonBoth_4_2_3\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D7375D4-166E-4193-A5B5-6D218E46FB9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F91AD356-F795-436E-BACE-9791635FBCA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D93492AF-A3DE-408F-9435-2890689047C1}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="49">
   <si>
     <t>HEATPUMPRX</t>
   </si>
@@ -141,18 +141,6 @@
     <t>gpio.h</t>
   </si>
   <si>
-    <t>src\HeishaMonBoth.cpp</t>
-  </si>
-  <si>
-    <t>\dallas.h</t>
-  </si>
-  <si>
-    <t>\HeishaOT.h</t>
-  </si>
-  <si>
-    <t>\s0.cpp</t>
-  </si>
-  <si>
     <t>Files setting</t>
   </si>
   <si>
@@ -165,9 +153,6 @@
     <t>modbusTxPin</t>
   </si>
   <si>
-    <t>\rs485modbus.h</t>
-  </si>
-  <si>
     <t>GPIO New</t>
   </si>
   <si>
@@ -184,6 +169,18 @@
   </si>
   <si>
     <t>Input only</t>
+  </si>
+  <si>
+    <t>HeishaMonBoth.cpp</t>
+  </si>
+  <si>
+    <t>s0.cpp</t>
+  </si>
+  <si>
+    <t>dallas.h</t>
+  </si>
+  <si>
+    <t>HeishaOT.h</t>
   </si>
 </sst>
 </file>
@@ -339,7 +336,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -421,6 +418,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -751,25 +751,25 @@
     <row r="1" spans="1:8" s="15" customFormat="1" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="14"/>
       <c r="B1" s="12" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="G1" s="14" t="s">
         <v>33</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
@@ -783,7 +783,7 @@
         <v>4</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E2" s="6">
         <v>0</v>
@@ -847,7 +847,7 @@
         <v>15</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="17"/>
@@ -869,7 +869,7 @@
         <v>23</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="17"/>
@@ -975,7 +975,7 @@
         <v>9</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E14" s="6">
         <v>12</v>
@@ -1013,7 +1013,7 @@
         <v>10</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E16" s="3">
         <v>14</v>
@@ -1039,10 +1039,14 @@
         <v>25</v>
       </c>
       <c r="D17" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E17" s="30">
+        <v>15</v>
+      </c>
+      <c r="F17" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="E17" s="3"/>
-      <c r="F17" s="17"/>
       <c r="G17" s="5">
         <v>15</v>
       </c>
@@ -1059,7 +1063,7 @@
         <v>1</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E18" s="9">
         <v>16</v>
@@ -1079,7 +1083,7 @@
         <v>0</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E19" s="9">
         <v>17</v>
@@ -1146,15 +1150,17 @@
         <v>21</v>
       </c>
       <c r="C22" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E22" s="3">
+        <v>38</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="E22" s="30">
         <v>21</v>
       </c>
-      <c r="F22" s="17"/>
+      <c r="F22" s="29" t="s">
+        <v>37</v>
+      </c>
       <c r="G22" s="5">
         <v>21</v>
       </c>
@@ -1171,7 +1177,7 @@
         <v>26</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E23" s="26">
         <v>22</v>
@@ -1190,10 +1196,10 @@
         <v>23</v>
       </c>
       <c r="C24" s="29" t="s">
-        <v>41</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>43</v>
+        <v>37</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>45</v>
       </c>
       <c r="E24" s="26">
         <v>23</v>
@@ -1213,7 +1219,7 @@
         <v>14</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E25" s="3">
         <v>25</v>
@@ -1233,7 +1239,7 @@
         <v>2</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E26" s="9">
         <v>26</v>
@@ -1253,7 +1259,7 @@
         <v>3</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E27" s="9">
         <v>27</v>
@@ -1273,7 +1279,7 @@
         <v>24</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="E28" s="3">
         <v>32</v>
@@ -1295,7 +1301,7 @@
         <v>13</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E29" s="3">
         <v>33</v>
@@ -1308,7 +1314,7 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B30" s="8">
         <v>34</v>
@@ -1317,7 +1323,7 @@
         <v>11</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E30" s="8">
         <v>34</v>
@@ -1330,43 +1336,49 @@
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B31" s="8">
         <v>35</v>
       </c>
       <c r="C31" s="24" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E31" s="8">
         <v>35</v>
       </c>
       <c r="F31" s="17" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="G31" s="5"/>
       <c r="H31" s="17"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B32" s="8">
         <v>36</v>
       </c>
       <c r="C32" s="17"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="17"/>
+      <c r="D32" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E32" s="26">
+        <v>36</v>
+      </c>
+      <c r="F32" s="25" t="s">
+        <v>6</v>
+      </c>
       <c r="G32" s="5"/>
       <c r="H32" s="17"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B33" s="8">
         <v>39</v>
@@ -1375,7 +1387,7 @@
         <v>22</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="E33" s="3"/>
       <c r="F33" s="17"/>

</xml_diff>